<commit_message>
Fix typed player counts in the rank distribution workbook
Players_int no longer matched the Players column it was typed from in 34 KR,
22 BR and 2 EUNE cells (e.g. KR Bronze IV 105K as 1,051,056, BR divisions
pasted as 15,000, EUNE Grandmaster 539 as 539,000), which made the EUNE tier
shares sum to 154.8%. The cells now hold the Players value, as on the EUW
and NA sheets, and Excel recalculates the side tables on open. EUW and NA
are unchanged. With correct totals KR's fetch plan sums to 2,797 instead of
2,800, as Bronze, Silver and Gold each drop by one.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/ANALYSIS/data/LoL Rank Distribution via DPM.LOL.xlsx
+++ b/src/ANALYSIS/data/LoL Rank Distribution via DPM.LOL.xlsx
@@ -20,7 +20,7 @@
     <sheet name="EUNE" sheetId="4" r:id="rId5"/>
     <sheet name="BR" sheetId="2" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -3891,7 +3891,7 @@
         <v>15</v>
       </c>
       <c r="I3">
-        <v>10109</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
@@ -3920,7 +3920,7 @@
         <v>15</v>
       </c>
       <c r="I4">
-        <v>23239</v>
+        <v>23000</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
@@ -3949,7 +3949,7 @@
         <v>15</v>
       </c>
       <c r="I5">
-        <v>61618</v>
+        <v>61000</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
@@ -3978,7 +3978,7 @@
         <v>246</v>
       </c>
       <c r="I6">
-        <v>104104</v>
+        <v>104000</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
@@ -4007,7 +4007,7 @@
         <v>15</v>
       </c>
       <c r="I7">
-        <v>1051056</v>
+        <v>105000</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
@@ -4036,7 +4036,7 @@
         <v>15</v>
       </c>
       <c r="I8">
-        <v>93932</v>
+        <v>93000</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
@@ -4065,7 +4065,7 @@
         <v>15</v>
       </c>
       <c r="I9">
-        <v>1011018</v>
+        <v>101000</v>
       </c>
       <c r="L9" t="s">
         <v>601</v>
@@ -4115,7 +4115,7 @@
         <v>15</v>
       </c>
       <c r="I10">
-        <v>97974</v>
+        <v>97000</v>
       </c>
       <c r="L10">
         <v>2623034</v>
@@ -4128,11 +4128,11 @@
       </c>
       <c r="O10">
         <f>I6</f>
-        <v>104104</v>
+        <v>104000</v>
       </c>
       <c r="P10">
         <f t="shared" ref="P10:P19" si="0">(O10/$L$10*100)</f>
-        <v>3.9688391381888302</v>
+        <v>3.964874263924905</v>
       </c>
       <c r="Q10">
         <f>INT($M$10*(P10/100))</f>
@@ -4140,7 +4140,7 @@
       </c>
       <c r="R10">
         <f>SUM(Q10:Q19)</f>
-        <v>2800</v>
+        <v>2797</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
@@ -4169,22 +4169,22 @@
         <v>211</v>
       </c>
       <c r="I11">
-        <v>395395</v>
+        <v>395000</v>
       </c>
       <c r="N11" t="s">
         <v>37</v>
       </c>
       <c r="O11">
         <f>I11</f>
-        <v>395395</v>
+        <v>395000</v>
       </c>
       <c r="P11">
         <f t="shared" si="0"/>
-        <v>15.0739563421595</v>
+        <v>15.058897444714784</v>
       </c>
       <c r="Q11">
         <f t="shared" ref="Q11:Q17" si="1">INT($M$10*(P11/100))</f>
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
@@ -4213,22 +4213,22 @@
         <v>15</v>
       </c>
       <c r="I12">
-        <v>1681681</v>
+        <v>168000</v>
       </c>
       <c r="N12" t="s">
         <v>60</v>
       </c>
       <c r="O12">
         <f>I16</f>
-        <v>577577</v>
+        <v>577000</v>
       </c>
       <c r="P12">
         <f t="shared" si="0"/>
-        <v>22.019424833989952</v>
+        <v>21.99742740658337</v>
       </c>
       <c r="Q12">
         <f t="shared" si="1"/>
-        <v>616</v>
+        <v>615</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
@@ -4257,22 +4257,22 @@
         <v>15</v>
       </c>
       <c r="I13">
-        <v>1461464</v>
+        <v>146000</v>
       </c>
       <c r="N13" t="s">
         <v>83</v>
       </c>
       <c r="O13">
         <f>I21</f>
-        <v>621621</v>
+        <v>621000</v>
       </c>
       <c r="P13">
         <f t="shared" si="0"/>
-        <v>23.698549084762149</v>
+        <v>23.674874210551597</v>
       </c>
       <c r="Q13">
         <f t="shared" si="1"/>
-        <v>663</v>
+        <v>662</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
@@ -4301,18 +4301,18 @@
         <v>15</v>
       </c>
       <c r="I14">
-        <v>1451459</v>
+        <v>145000</v>
       </c>
       <c r="N14" t="s">
         <v>99</v>
       </c>
       <c r="O14">
         <f>I26</f>
-        <v>465465</v>
+        <v>465000</v>
       </c>
       <c r="P14">
         <f t="shared" si="0"/>
-        <v>17.745290377478902</v>
+        <v>17.727562814664243</v>
       </c>
       <c r="Q14">
         <f t="shared" si="1"/>
@@ -4345,18 +4345,18 @@
         <v>15</v>
       </c>
       <c r="I15">
-        <v>1181183</v>
+        <v>118000</v>
       </c>
       <c r="N15" t="s">
         <v>118</v>
       </c>
       <c r="O15">
         <f>I31</f>
-        <v>298298</v>
+        <v>298000</v>
       </c>
       <c r="P15">
         <f t="shared" si="0"/>
-        <v>11.372250607502609</v>
+        <v>11.360889717784826</v>
       </c>
       <c r="Q15">
         <f t="shared" si="1"/>
@@ -4389,18 +4389,18 @@
         <v>349</v>
       </c>
       <c r="I16">
-        <v>577577</v>
+        <v>577000</v>
       </c>
       <c r="N16" t="s">
         <v>139</v>
       </c>
       <c r="O16">
         <f>I36</f>
-        <v>138138</v>
+        <v>138000</v>
       </c>
       <c r="P16">
         <f t="shared" si="0"/>
-        <v>5.2663442410582553</v>
+        <v>5.261083157900355</v>
       </c>
       <c r="Q16">
         <f t="shared" si="1"/>
@@ -4433,7 +4433,7 @@
         <v>15</v>
       </c>
       <c r="I17">
-        <v>2222229</v>
+        <v>222000</v>
       </c>
       <c r="N17" t="s">
         <v>160</v>
@@ -4477,7 +4477,7 @@
         <v>15</v>
       </c>
       <c r="I18">
-        <v>1581580</v>
+        <v>158000</v>
       </c>
       <c r="N18" t="s">
         <v>167</v>
@@ -4520,7 +4520,7 @@
         <v>15</v>
       </c>
       <c r="I19">
-        <v>1411414</v>
+        <v>141000</v>
       </c>
       <c r="N19" t="s">
         <v>172</v>
@@ -4563,7 +4563,7 @@
         <v>15</v>
       </c>
       <c r="I20">
-        <v>1001009</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.25">
@@ -4592,7 +4592,7 @@
         <v>260</v>
       </c>
       <c r="I21">
-        <v>621621</v>
+        <v>621000</v>
       </c>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.25">
@@ -4621,7 +4621,7 @@
         <v>15</v>
       </c>
       <c r="I22">
-        <v>1931935</v>
+        <v>193000</v>
       </c>
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.25">
@@ -4650,7 +4650,7 @@
         <v>15</v>
       </c>
       <c r="I23">
-        <v>1171178</v>
+        <v>117000</v>
       </c>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.25">
@@ -4679,7 +4679,7 @@
         <v>15</v>
       </c>
       <c r="I24">
-        <v>94943</v>
+        <v>94000</v>
       </c>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.25">
@@ -4708,7 +4708,7 @@
         <v>15</v>
       </c>
       <c r="I25">
-        <v>61619</v>
+        <v>61000</v>
       </c>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.25">
@@ -4737,7 +4737,7 @@
         <v>378</v>
       </c>
       <c r="I26">
-        <v>465465</v>
+        <v>465000</v>
       </c>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.25">
@@ -4766,7 +4766,7 @@
         <v>15</v>
       </c>
       <c r="I27">
-        <v>1161167</v>
+        <v>116000</v>
       </c>
     </row>
     <row r="28" spans="1:17" x14ac:dyDescent="0.25">
@@ -4795,7 +4795,7 @@
         <v>15</v>
       </c>
       <c r="I28">
-        <v>47473</v>
+        <v>47000</v>
       </c>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.25">
@@ -4824,7 +4824,7 @@
         <v>15</v>
       </c>
       <c r="I29">
-        <v>93931</v>
+        <v>93000</v>
       </c>
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.25">
@@ -4853,7 +4853,7 @@
         <v>15</v>
       </c>
       <c r="I30">
-        <v>4242</v>
+        <v>42000</v>
       </c>
     </row>
     <row r="31" spans="1:17" x14ac:dyDescent="0.25">
@@ -4882,7 +4882,7 @@
         <v>390</v>
       </c>
       <c r="I31">
-        <v>298298</v>
+        <v>298000</v>
       </c>
     </row>
     <row r="32" spans="1:17" x14ac:dyDescent="0.25">
@@ -4911,7 +4911,7 @@
         <v>15</v>
       </c>
       <c r="I32">
-        <v>6868</v>
+        <v>68000</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
@@ -4940,7 +4940,7 @@
         <v>15</v>
       </c>
       <c r="I33">
-        <v>1717</v>
+        <v>17000</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -4969,7 +4969,7 @@
         <v>15</v>
       </c>
       <c r="I34">
-        <v>3030</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -4998,7 +4998,7 @@
         <v>15</v>
       </c>
       <c r="I35">
-        <v>2323</v>
+        <v>23000</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -5027,7 +5027,7 @@
         <v>399</v>
       </c>
       <c r="I36">
-        <v>138138</v>
+        <v>138000</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -7145,11 +7145,11 @@
       </c>
       <c r="O18">
         <f>I38</f>
-        <v>539000</v>
+        <v>539</v>
       </c>
       <c r="P18">
         <f t="shared" si="0"/>
-        <v>39.851123890416062</v>
+        <v>0.03985112389041606</v>
       </c>
       <c r="Q18">
         <v>3</v>
@@ -7188,11 +7188,11 @@
       </c>
       <c r="O19">
         <f>I39</f>
-        <v>202000</v>
+        <v>202</v>
       </c>
       <c r="P19">
         <f t="shared" si="0"/>
-        <v>14.934929547057596</v>
+        <v>0.014934929547057597</v>
       </c>
       <c r="Q19">
         <v>2</v>
@@ -7746,7 +7746,7 @@
         <v>403</v>
       </c>
       <c r="I38">
-        <v>539000</v>
+        <v>539</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -7775,7 +7775,7 @@
         <v>406</v>
       </c>
       <c r="I39">
-        <v>202000</v>
+        <v>202</v>
       </c>
     </row>
   </sheetData>
@@ -7996,7 +7996,7 @@
         <v>15</v>
       </c>
       <c r="I7">
-        <v>15000</v>
+        <v>44000</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
@@ -8025,7 +8025,7 @@
         <v>15</v>
       </c>
       <c r="I8">
-        <v>15000</v>
+        <v>38000</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
@@ -8054,7 +8054,7 @@
         <v>15</v>
       </c>
       <c r="I9">
-        <v>15000</v>
+        <v>42000</v>
       </c>
       <c r="L9" t="s">
         <v>601</v>
@@ -8104,7 +8104,7 @@
         <v>15</v>
       </c>
       <c r="I10">
-        <v>15000</v>
+        <v>46000</v>
       </c>
       <c r="L10">
         <v>1054597</v>
@@ -8202,7 +8202,7 @@
         <v>15</v>
       </c>
       <c r="I12">
-        <v>15000</v>
+        <v>50000</v>
       </c>
       <c r="N12" t="s">
         <v>60</v>
@@ -8246,7 +8246,7 @@
         <v>15</v>
       </c>
       <c r="I13">
-        <v>15000</v>
+        <v>65000</v>
       </c>
       <c r="N13" t="s">
         <v>83</v>
@@ -8290,7 +8290,7 @@
         <v>15</v>
       </c>
       <c r="I14">
-        <v>15000</v>
+        <v>60000</v>
       </c>
       <c r="N14" t="s">
         <v>99</v>
@@ -8334,7 +8334,7 @@
         <v>15</v>
       </c>
       <c r="I15">
-        <v>15000</v>
+        <v>66000</v>
       </c>
       <c r="N15" t="s">
         <v>118</v>
@@ -8422,7 +8422,7 @@
         <v>15</v>
       </c>
       <c r="I17">
-        <v>15000</v>
+        <v>67000</v>
       </c>
       <c r="N17" t="s">
         <v>160</v>
@@ -8466,7 +8466,7 @@
         <v>15</v>
       </c>
       <c r="I18">
-        <v>15000</v>
+        <v>60000</v>
       </c>
       <c r="N18" t="s">
         <v>167</v>
@@ -8509,7 +8509,7 @@
         <v>15</v>
       </c>
       <c r="I19">
-        <v>15000</v>
+        <v>66000</v>
       </c>
       <c r="N19" t="s">
         <v>172</v>
@@ -8552,7 +8552,7 @@
         <v>15</v>
       </c>
       <c r="I20">
-        <v>15000</v>
+        <v>55000</v>
       </c>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.25">
@@ -8610,7 +8610,7 @@
         <v>15</v>
       </c>
       <c r="I22">
-        <v>15000</v>
+        <v>54000</v>
       </c>
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.25">
@@ -8639,7 +8639,7 @@
         <v>15</v>
       </c>
       <c r="I23">
-        <v>15000</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.25">
@@ -8668,7 +8668,7 @@
         <v>15</v>
       </c>
       <c r="I24">
-        <v>15000</v>
+        <v>41000</v>
       </c>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.25">
@@ -8697,7 +8697,7 @@
         <v>15</v>
       </c>
       <c r="I25">
-        <v>15000</v>
+        <v>28000</v>
       </c>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.25">
@@ -8755,7 +8755,7 @@
         <v>15</v>
       </c>
       <c r="I27">
-        <v>15000</v>
+        <v>53000</v>
       </c>
     </row>
     <row r="28" spans="1:17" x14ac:dyDescent="0.25">
@@ -8784,7 +8784,7 @@
         <v>15</v>
       </c>
       <c r="I28">
-        <v>15000</v>
+        <v>29000</v>
       </c>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.25">
@@ -8813,7 +8813,7 @@
         <v>15</v>
       </c>
       <c r="I29">
-        <v>15000</v>
+        <v>21000</v>
       </c>
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.25">
@@ -8842,7 +8842,7 @@
         <v>15</v>
       </c>
       <c r="I30">
-        <v>15000</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="31" spans="1:17" x14ac:dyDescent="0.25">
@@ -8900,7 +8900,7 @@
         <v>15</v>
       </c>
       <c r="I32">
-        <v>15000</v>
+        <v>16000</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
@@ -8958,7 +8958,7 @@
         <v>15</v>
       </c>
       <c r="I34">
-        <v>15000</v>
+        <v>11000</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">

</xml_diff>